<commit_message>
LTS1: evidenceCondition applied_pressure; properties modulus_youngs bound to PerformanceCriterion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/evidenceCondition.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/evidenceCondition.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ValueBindings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Lists" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ValueBindings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1000,7 +1000,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,36 @@
         <f>IF(ISNA(VLOOKUP(B4,AssociatedElements!B$2:B2942,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="G4" s="9" t="n"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>applied_pressure</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Applied pressure</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The pressure applied to the test surface at which a measured response is read - for example the 150 kPa design pressure at which the settlement under a plate or zone load test is judged. Restricts the evidence of a criterion to readings taken at that applied pressure.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2">
@@ -1628,7 +1657,21 @@
         <f>IF(ISNA(VLOOKUP(B4,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>applied_pressure</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>//diggs:parameterName</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:evidenceCondition</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5">

</xml_diff>